<commit_message>
feat: add cargo de confiança functionality to import and calculation processes
</commit_message>
<xml_diff>
--- a/app/public/modelos/modelo-nome.xlsx
+++ b/app/public/modelos/modelo-nome.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Funcionarios" sheetId="1" r:id="rId1"/>
+    <sheet name="Dados" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,13 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,6 +412,9 @@
       <c r="D1" t="str">
         <v>TIPO</v>
       </c>
+      <c r="E1" t="str">
+        <v>CARGO_CONFIANCA</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,6 +429,9 @@
       <c r="D2" t="str">
         <v>CLT</v>
       </c>
+      <c r="E2" t="str">
+        <v>NAO</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -446,6 +446,9 @@
       <c r="D3" t="str">
         <v>CLT</v>
       </c>
+      <c r="E3" t="str">
+        <v>SIM</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -460,6 +463,9 @@
       <c r="D4" t="str">
         <v>CLT</v>
       </c>
+      <c r="E4" t="str">
+        <v>NAO</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -474,6 +480,9 @@
       <c r="D5" t="str">
         <v>CLT</v>
       </c>
+      <c r="E5" t="str">
+        <v>NAO</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -488,6 +497,9 @@
       <c r="D6" t="str">
         <v>PCD</v>
       </c>
+      <c r="E6" t="str">
+        <v>NAO</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -502,6 +514,9 @@
       <c r="D7" t="str">
         <v>APRENDIZ</v>
       </c>
+      <c r="E7" t="str">
+        <v>NAO</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -516,6 +531,9 @@
       <c r="D8" t="str">
         <v>ESTAGIARIO</v>
       </c>
+      <c r="E8" t="str">
+        <v>NAO</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -530,10 +548,13 @@
       <c r="D9" t="str">
         <v>CLT</v>
       </c>
+      <c r="E9" t="str">
+        <v>NAO</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: removed Cargo de Confianca and added Afastado pelo INSS, Terceirizado, Trabalhador Temporario
</commit_message>
<xml_diff>
--- a/app/public/modelos/modelo-nome.xlsx
+++ b/app/public/modelos/modelo-nome.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,9 +412,6 @@
       <c r="D1" t="str">
         <v>TIPO</v>
       </c>
-      <c r="E1" t="str">
-        <v>CARGO_CONFIANCA</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -429,9 +426,6 @@
       <c r="D2" t="str">
         <v>CLT</v>
       </c>
-      <c r="E2" t="str">
-        <v>NAO</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -446,9 +440,6 @@
       <c r="D3" t="str">
         <v>CLT</v>
       </c>
-      <c r="E3" t="str">
-        <v>SIM</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -463,9 +454,6 @@
       <c r="D4" t="str">
         <v>CLT</v>
       </c>
-      <c r="E4" t="str">
-        <v>NAO</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -480,9 +468,6 @@
       <c r="D5" t="str">
         <v>CLT</v>
       </c>
-      <c r="E5" t="str">
-        <v>NAO</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -495,10 +480,7 @@
         <v>411010</v>
       </c>
       <c r="D6" t="str">
-        <v>CLT</v>
-      </c>
-      <c r="E6" t="str">
-        <v>NAO</v>
+        <v>AFASTADO PELO INSS</v>
       </c>
     </row>
     <row r="7">
@@ -514,25 +496,19 @@
       <c r="D7" t="str">
         <v>APRENDIZ</v>
       </c>
-      <c r="E7" t="str">
-        <v>NAO</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>11.111.111/0002-22</v>
+        <v>11.111.111/0001-11</v>
       </c>
       <c r="B8" t="str">
-        <v>Fabio Melo</v>
+        <v>Igor Prado</v>
       </c>
       <c r="C8" t="str">
-        <v>351305</v>
+        <v>514320</v>
       </c>
       <c r="D8" t="str">
-        <v>ESTAGIARIO</v>
-      </c>
-      <c r="E8" t="str">
-        <v>NAO</v>
+        <v>TERCEIRIZADO</v>
       </c>
     </row>
     <row r="9">
@@ -540,21 +516,46 @@
         <v>11.111.111/0002-22</v>
       </c>
       <c r="B9" t="str">
+        <v>Fabio Melo</v>
+      </c>
+      <c r="C9" t="str">
+        <v>351305</v>
+      </c>
+      <c r="D9" t="str">
+        <v>ESTAGIARIO</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>11.111.111/0002-22</v>
+      </c>
+      <c r="B10" t="str">
         <v>Helena Cruz</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C10" t="str">
         <v>411010</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D10" t="str">
         <v>CLT</v>
       </c>
-      <c r="E9" t="str">
-        <v>NAO</v>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>11.111.111/0002-22</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Joana Reis</v>
+      </c>
+      <c r="C11" t="str">
+        <v>411010</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TRABALHO TEMPORARIO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>